<commit_message>
Correct received spring length to owner-confirmed 50 mm
</commit_message>
<xml_diff>
--- a/procurement/mode_a_procurement_bom_2026-08-21.xlsx
+++ b/procurement/mode_a_procurement_bom_2026-08-21.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rd364db9636ea4dcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R1d284126e4e346ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="R7bc753c6ff774762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="Rfb05944210a345ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="R5156f58c0c884f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="Recbfcf38629e457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R7a8f7a8a49174c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="Rd26c604b2d6c49ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="Refd93be5c4d44447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R25c4ac21fb914445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="Rf79779430ebf4978"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="R23e956d44e3749db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="Rb08b1807cf7e4b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="Rf1e99c1512f04f10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="R2b230ada690040fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R0f749c71e06141a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="R2cec2c7177754d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="Ra3d9622be4b64a73"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,9 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="202" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="59">
     <x:font>
@@ -363,7 +364,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="26">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -488,6 +489,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F3EC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -679,7 +685,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="284">
+  <x:cellXfs count="290">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1358,6 +1364,20 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="54" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="54" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1743,10 +1763,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B11" s="168" t="str">
-        <x:v>Resolve the five exact RFQs</x:v>
+        <x:v>Resolve remaining fit and CAD work</x:v>
       </x:c>
       <x:c r="C11" s="169" t="str">
-        <x:v>Spring, Ø10 knee axle, Ø6 stop pin, Ø5 guide shaft and Ø19/13.6 shims. For the knee axle, do not accept a common m6 dowel; require h6 or a verified tighter h5 shaft.</x:v>
+        <x:v>The yellow OD18 / ID9 x 50 mm spring is owned. Adapt the cartridge, then verify its rate. The knee axle, stop pin, guide shaft and preload hardware retain their separate fit/design gates.</x:v>
       </x:c>
       <x:c r="D11" s="147"/>
       <x:c r="E11" s="147"/>
@@ -3563,9 +3583,9 @@
         <x:v>Release evidence</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="5" ht="72" hidden="0" customHeight="1">
       <x:c r="A5" s="183" t="str">
-        <x:v>RFQ now</x:v>
+        <x:v>Owned; adapt CAD</x:v>
       </x:c>
       <x:c r="B5" s="176" t="str">
         <x:v>Spring</x:v>
@@ -3574,25 +3594,25 @@
         <x:v>Knee compression spring</x:v>
       </x:c>
       <x:c r="D5" s="176" t="str">
-        <x:v>OD 19 mm; wire 2.6 mm; free length 55 mm; closed &amp; ground; chrome-silicon ASTM A877/A877M; shot-peened + preset; rate 10.45 N/mm ±5%; ~9.8 active coils. A228 music wire acceptable for early prototype only.</x:v>
+        <x:v>Owned: Yellow TF, OD18 / ID9 x 50 mm free. Owner confirmed 5 cm on 2026-09-06. Original 55 mm CAD baseline remains unadapted. Actual rate unverified.</x:v>
       </x:c>
       <x:c r="E5" s="176" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="176" t="str">
-        <x:v>Send the exact specification to local Santa Clara/San Jose spring shops and request one prototype plus price breaks for 2 and 5.</x:v>
+        <x:v>Keep the owned spring. Adapt seats, installed length and internal stop/bumper in Fusion. No replacement for length is needed.</x:v>
       </x:c>
       <x:c r="G5" s="178" t="str">
-        <x:v>American Precision Spring</x:v>
+        <x:v>Original 55 mm RFQ: American Precision Spring</x:v>
       </x:c>
       <x:c r="H5" s="178" t="str">
-        <x:v>APS San Jose</x:v>
+        <x:v>Original 55 mm RFQ: APS San Jose</x:v>
       </x:c>
       <x:c r="I5" s="176" t="str">
-        <x:v>No exact stock spring was found. Rate/material/process matter to both travel and load.</x:v>
+        <x:v>CAD has diameter 13.4 spigots, 10 washer stack and 13 bumper. These do not fit the owned spring ID9.</x:v>
       </x:c>
       <x:c r="J5" s="176" t="str">
-        <x:v>Supplier drawing + measured free length and rate acceptance.</x:v>
+        <x:v>Order screenshot confirms Yellow / 50 mm / OD18 / ID9. Owner confirmed received length on 2026-09-06. CAD adaptation and rate acceptance pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -4463,6 +4483,26 @@
         <x:v>Fit the exact insert in the Ø4.0 × 5.0 ABS coupon; reserve 14 for the active build.</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="72" customHeight="1">
+      <x:c r="A20" s="288" t="str">
+        <x:v>Owned</x:v>
+      </x:c>
+      <x:c r="B20" s="288" t="str">
+        <x:v>Spring</x:v>
+      </x:c>
+      <x:c r="C20" s="288" t="str">
+        <x:v>Yellow TF, OD18 / ID9 x 50 mm free</x:v>
+      </x:c>
+      <x:c r="D20" s="289" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="288" t="str">
+        <x:v>https://github.com/TnnsBeast/Biped/tree/main/evidence/springs/2026-09-05_reconciliation</x:v>
+      </x:c>
+      <x:c r="F20" s="288" t="str">
+        <x:v>Owner confirms 5 cm. Keep this spring. Cartridge adaptation and measured rate remain open.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -4800,7 +4840,7 @@
         <x:v>Local spring shops</x:v>
       </x:c>
       <x:c r="C18" s="176" t="str">
-        <x:v>Custom compression-spring RFQ paths in Santa Clara/San Jose</x:v>
+        <x:v>Original 55 mm spring RFQ paths (deferred)</x:v>
       </x:c>
       <x:c r="D18" s="191" t="n">
         <x:v>46255</x:v>
@@ -5524,12 +5564,12 @@
         <x:v>Conditional row 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
+    <x:row r="35" ht="42" hidden="0" customHeight="1">
       <x:c r="A35" s="176" t="str">
-        <x:v>RFQ now</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="B35" s="176" t="str">
-        <x:v>Knee compression spring</x:v>
+        <x:v>Knee spring: original 55 mm RFQ (deferred)</x:v>
       </x:c>
       <x:c r="C35" s="176" t="str">
         <x:v>American Precision Spring</x:v>
@@ -5538,7 +5578,7 @@
         <x:v>https://americanprecspring.com/</x:v>
       </x:c>
       <x:c r="E35" s="176" t="str">
-        <x:v>RFQ &amp; Holds row 5</x:v>
+        <x:v>Keep the owned 50 mm spring. Baseline supplier reference only.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -5609,12 +5649,12 @@
         <x:v>RFQ &amp; Holds row 9</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="15" hidden="0" customHeight="1">
+    <x:row r="40" ht="42" hidden="0" customHeight="1">
       <x:c r="A40" s="176" t="str">
-        <x:v>RFQ fallback</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="B40" s="176" t="str">
-        <x:v>Knee compression spring</x:v>
+        <x:v>Knee spring: original 55 mm RFQ (deferred)</x:v>
       </x:c>
       <x:c r="C40" s="176" t="str">
         <x:v>Advanced Precision Spring — San Jose</x:v>
@@ -5623,7 +5663,7 @@
         <x:v>https://apspring.com/</x:v>
       </x:c>
       <x:c r="E40" s="176" t="str">
-        <x:v>Local fallback</x:v>
+        <x:v>Keep the owned 50 mm spring. Baseline supplier reference only.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -6042,28 +6082,28 @@
         <x:v>Mechanical assembly</x:v>
       </x:c>
       <x:c r="B16" s="246" t="str">
-        <x:v>OPEN / RFQ</x:v>
+        <x:v>SPRING OWNED; ADAPT CAD</x:v>
       </x:c>
       <x:c r="C16" s="243" t="str">
-        <x:v>Main spring, Ø6 h6 stop pin, Ø5 h6 guide shaft, Ø19/Ø13.6 preload shims</x:v>
+        <x:v>Owned 50 mm spring; stop pin, guide shaft and revised preload hardware remain open.</x:v>
       </x:c>
       <x:c r="D16" s="243" t="str">
         <x:v>RFQ &amp; Holds rows 5, 7–9</x:v>
       </x:c>
       <x:c r="E16" s="243" t="str">
-        <x:v>Complete ABS single-leg fit, assembly, wiring, and unloaded controls integration; leave the main spring unpreloaded and structural-load fixtures unused.</x:v>
+        <x:v>Adapt the cartridge to the owned Yellow OD18 / ID9 x 50 mm spring. Continue springless ABS fit and hand assembly until the cartridge is verified.</x:v>
       </x:c>
       <x:c r="F16" s="243" t="str">
-        <x:v>Geometry and wheel-clear/current-limited self-weight checks only.</x:v>
+        <x:v>The spring length is confirmed. Seats and internal stop/bumper still require redesign and rate verification.</x:v>
       </x:c>
       <x:c r="G16" s="243" t="str">
         <x:v>Active now through unloaded single-leg commissioning.</x:v>
       </x:c>
       <x:c r="H16" s="243" t="str">
-        <x:v>No torque-arm, main-spring, ground-traction, stall/proof, drop, or human-adjacent loading in ABS.</x:v>
+        <x:v>Keep the owned spring; no replacement for length is needed. No spring preload or structural loads through ABS.</x:v>
       </x:c>
       <x:c r="I16" s="243" t="str">
-        <x:v>beni_single_leg_rig_design_record.md §9</x:v>
+        <x:v>https://github.com/TnnsBeast/Biped/tree/main/evidence/springs/2026-09-05_reconciliation</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="57" customHeight="1">
@@ -6249,8 +6289,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876452d0a3dd4285"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf8ee2b37a6943a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46d1c0d416b45f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fa43da2da494a0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>